<commit_message>
ajustes baseado na atualização das bases
bases foram alteradas e o código foi adaptado para a nova estrutura
</commit_message>
<xml_diff>
--- a/reports/dic_colunas_complemento.xlsx
+++ b/reports/dic_colunas_complemento.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C245"/>
+  <dimension ref="A1:C255"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3129,6 +3129,116 @@
       </c>
       <c r="C245" t="inlineStr"/>
     </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>fg_ativo</t>
+        </is>
+      </c>
+      <c r="B246" t="n">
+        <v>0</v>
+      </c>
+      <c r="C246" t="inlineStr"/>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>fg_status_vol_3m</t>
+        </is>
+      </c>
+      <c r="B247" t="n">
+        <v>0</v>
+      </c>
+      <c r="C247" t="inlineStr"/>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>fg_status_vol_5m</t>
+        </is>
+      </c>
+      <c r="B248" t="n">
+        <v>0</v>
+      </c>
+      <c r="C248" t="inlineStr"/>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>fg_status_vol_6m</t>
+        </is>
+      </c>
+      <c r="B249" t="n">
+        <v>0</v>
+      </c>
+      <c r="C249" t="inlineStr"/>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>fg_status_vol_7m</t>
+        </is>
+      </c>
+      <c r="B250" t="n">
+        <v>0</v>
+      </c>
+      <c r="C250" t="inlineStr"/>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>fg_status_vol_8m</t>
+        </is>
+      </c>
+      <c r="B251" t="n">
+        <v>0</v>
+      </c>
+      <c r="C251" t="inlineStr"/>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>fg_status_vol_9m</t>
+        </is>
+      </c>
+      <c r="B252" t="n">
+        <v>0</v>
+      </c>
+      <c r="C252" t="inlineStr"/>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>fg_status_vol_10m</t>
+        </is>
+      </c>
+      <c r="B253" t="n">
+        <v>0</v>
+      </c>
+      <c r="C253" t="inlineStr"/>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>fg_status_vol_11m</t>
+        </is>
+      </c>
+      <c r="B254" t="n">
+        <v>0</v>
+      </c>
+      <c r="C254" t="inlineStr"/>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>fg_status_vol_12m</t>
+        </is>
+      </c>
+      <c r="B255" t="n">
+        <v>0</v>
+      </c>
+      <c r="C255" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
nova atualização da base
</commit_message>
<xml_diff>
--- a/reports/dic_colunas_complemento.xlsx
+++ b/reports/dic_colunas_complemento.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C255"/>
+  <dimension ref="A1:C268"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3239,6 +3239,149 @@
       </c>
       <c r="C255" t="inlineStr"/>
     </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>Benefício por Tempo 1_nzero_3m</t>
+        </is>
+      </c>
+      <c r="B256" t="n">
+        <v>0</v>
+      </c>
+      <c r="C256" t="inlineStr"/>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>Componente Variável 10_nzero_3m</t>
+        </is>
+      </c>
+      <c r="B257" t="n">
+        <v>0</v>
+      </c>
+      <c r="C257" t="inlineStr"/>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>Componente Variável 11_nzero_3m</t>
+        </is>
+      </c>
+      <c r="B258" t="n">
+        <v>0</v>
+      </c>
+      <c r="C258" t="inlineStr"/>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>Componente Variável 13_nzero_3m</t>
+        </is>
+      </c>
+      <c r="B259" t="n">
+        <v>0</v>
+      </c>
+      <c r="C259" t="inlineStr"/>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>Componente Variável 3_nzero_3m</t>
+        </is>
+      </c>
+      <c r="B260" t="n">
+        <v>0</v>
+      </c>
+      <c r="C260" t="inlineStr"/>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>Componente Variável 5_nzero_3m</t>
+        </is>
+      </c>
+      <c r="B261" t="n">
+        <v>0</v>
+      </c>
+      <c r="C261" t="inlineStr"/>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>Componente Variável 6_nzero_3m</t>
+        </is>
+      </c>
+      <c r="B262" t="n">
+        <v>0</v>
+      </c>
+      <c r="C262" t="inlineStr"/>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>Componente Variável 7_nzero_3m</t>
+        </is>
+      </c>
+      <c r="B263" t="n">
+        <v>0</v>
+      </c>
+      <c r="C263" t="inlineStr"/>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>Componente Variável 8_nzero_3m</t>
+        </is>
+      </c>
+      <c r="B264" t="n">
+        <v>0</v>
+      </c>
+      <c r="C264" t="inlineStr"/>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>Componente Variável 9_nzero_3m</t>
+        </is>
+      </c>
+      <c r="B265" t="n">
+        <v>0</v>
+      </c>
+      <c r="C265" t="inlineStr"/>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>Insalubridade_nzero_3m</t>
+        </is>
+      </c>
+      <c r="B266" t="n">
+        <v>0</v>
+      </c>
+      <c r="C266" t="inlineStr"/>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>Salário substituição_nzero_3m</t>
+        </is>
+      </c>
+      <c r="B267" t="n">
+        <v>0</v>
+      </c>
+      <c r="C267" t="inlineStr"/>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>Sobreaviso_nzero_3m</t>
+        </is>
+      </c>
+      <c r="B268" t="n">
+        <v>0</v>
+      </c>
+      <c r="C268" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>